<commit_message>
Zaktualizowano plik Excel/Excel file updated
</commit_message>
<xml_diff>
--- a/Out4FunTestCases.xlsx
+++ b/Out4FunTestCases.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27813"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27909"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="227" documentId="11_9D5355BF84DCCE53631DEA188F31F45B3A7E0439" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{727002D3-E776-473F-BC12-6EB5C1DEF0EF}"/>
+  <xr:revisionPtr revIDLastSave="323" documentId="11_9D5355BF84DCCE53631DEA188F31F45B3A7E0439" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D75039E4-9632-4AFA-87E9-1D1A6226C776}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="92">
   <si>
     <t>Numer przypadku testowego:</t>
   </si>
@@ -239,17 +239,88 @@
     <t>Wskazywanie lokalizacji miejsca na mapie - zatwierdzanie współrzędnych.</t>
   </si>
   <si>
-    <t>Wskazać miejsce na mapie przez dwukrotne kliknięcie, wtedy wypełnią się pola na długość i szerokość geograficzną,</t>
+    <t>Wskazać miejsce na mapie przez dwukrotne kliknięcie, wtedy wypełnią się pola na długość i szerokość geograficzną.</t>
   </si>
   <si>
     <t>W polu Wskaż lokalizację miejsca na mapie, po każdorazowym kliknięciu na nowy punkt mapy, współrzędne powinny sie aktualizować.</t>
+  </si>
+  <si>
+    <t>16.</t>
+  </si>
+  <si>
+    <t>Dodawanie nowej atrakcji, puste pole "Rodzaj atrakcji".</t>
+  </si>
+  <si>
+    <t>Wypełnić wszystkie wymagane pola formularza, pomijając "Rodzaj atrakcji".</t>
+  </si>
+  <si>
+    <t>Wyświetla się komunikat: "Wybierz jedną z opcji z listy".</t>
+  </si>
+  <si>
+    <t>17.</t>
+  </si>
+  <si>
+    <t>Puste pole  lokalizacji miejsca na mapie.</t>
+  </si>
+  <si>
+    <t>Wypełnić wszystkie wymagane pola formularza, pomijając "Lokalizacja atrakcji".</t>
+  </si>
+  <si>
+    <t>Wyświetla się komunikat: "Brak współrzędnych atrakcji. Wymagana długość i szerokość geograficzna".</t>
+  </si>
+  <si>
+    <t>Pola długości i szerokości geograficznej są oznaczone zielonym znakiem "check". Atrakcja mimo to nie może zostać dodana. Brak komunikatu o błędzie.</t>
+  </si>
+  <si>
+    <t>18.</t>
+  </si>
+  <si>
+    <t>Wpisanie liter, zamiast współrzędnych atrakcji w polu "Lokalizacja atrakcji".</t>
+  </si>
+  <si>
+    <t>1. Wypełnić wszystkie wymagane pola formularza, przy czym  "Lokalizacja atrakcji" powinna zostać wypełniona przypadkowymi literami, np. "abcde".</t>
+  </si>
+  <si>
+    <t>Samo wpisanie jednego znaku, np. “a”, powoduje, iż strona nagle znika i widać tylko pustą stronę.</t>
+  </si>
+  <si>
+    <t>19.</t>
+  </si>
+  <si>
+    <t>Edytowanie istniejącego miejsca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Uruchomienie na pasku wyszukiwania przeglądarki Opera strony https://mydog-1247b.web.app.
+</t>
+  </si>
+  <si>
+    <t>1. Edytuj istniejące miejsce i zmień wszystkie pola, następnie zapisz zmiany.</t>
+  </si>
+  <si>
+    <t>Wyświetla się komunikat "Dziękujemy za rejestrację punktu na mapie.
+Punkt pojawi się na mapie gdy zostanie zatwierdzony przez osbługę." Po zatwierdzeniu atrakcji, jest ona widoczna na mapie.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taki sam, jak spodziewany. Warto jednak wziąć pod uwagę, iż poprzednio utworzona atrakcja nadal widnieje na mapie. </t>
+  </si>
+  <si>
+    <t>20.</t>
+  </si>
+  <si>
+    <t>Usunięcie z mapy istniejącego miejsca.</t>
+  </si>
+  <si>
+    <t>Opcja jest niedostępna dla zwykłego użytkownika.</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -264,6 +335,18 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Consolas"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -286,7 +369,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -299,6 +382,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -951,7 +1050,7 @@
       <c r="A16" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="4" t="s">
         <v>66</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -960,59 +1059,193 @@
       <c r="D16" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43.5" customHeight="1">
-      <c r="A17" s="1"/>
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="1"/>
-    </row>
-    <row r="21" spans="1:4">
-      <c r="A21" s="1"/>
-    </row>
-    <row r="22" spans="1:4">
-      <c r="A22" s="1"/>
-    </row>
-    <row r="23" spans="1:4">
+    <row r="17" spans="1:6" ht="43.5" customHeight="1">
+      <c r="A17" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="87">
+      <c r="A18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="43.5" customHeight="1">
+      <c r="A19" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="9"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="1:6" ht="72.75">
+      <c r="A21" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
       <c r="A23" s="1"/>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:6">
       <c r="A24" s="1"/>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="B24" s="7"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:6">
       <c r="A25" s="1"/>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+    </row>
+    <row r="26" spans="1:6">
       <c r="A26" s="1"/>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:6">
       <c r="A27" s="1"/>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" spans="1:6">
       <c r="A28" s="1"/>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6">
       <c r="A29" s="1"/>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6">
       <c r="A30" s="1"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D16:D17"/>
+  <mergeCells count="6">
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>